<commit_message>
README 9장 TC-63에 #15 원칙 추가, 엑셀 TC-63·71·77 메모 정리
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mini_hotel_test_cases_v2.xlsx
+++ b/docs/mini_hotel_test_cases_v2.xlsx
@@ -6109,7 +6109,8 @@
       <c r="M64" s="30" t="inlineStr">
         <is>
           <t>탐색 테스트. 메시지에 가입 경로(구글)가 노출되어 이메일만으로 가입 여부·가입 방법을 알 수 있음. 로그인 실패 메시지는 구분하지 않는 정책(TC-43)과 일관성 확인 필요
-[QA 정책 제안 2026-10-13, 확정 B] "이미 가입된 이메일입니다"만 표시하고 로그인 화면으로 안내 (가입 경로 숨김). 선택지: A 현행 유지(가입 경로 표시) / B 경로 숨김 / C 가입 여부도 숨김(이메일 인증 필요). 이유: 가입 경로 노출을 줄이면서 다음 행동은 안내, 로그인 실패 메시지 정책(TC-43)과 일관. 소셜 콜백 ACCOUNT_EXISTS의 provider 전달(명세 135행)도 함께 맞출 것</t>
+[QA 정책 제안 2026-10-13, 확정 B] "이미 가입된 이메일입니다"만 표시하고 로그인 화면으로 안내 (가입 경로 숨김). 선택지: A 현행 유지(가입 경로 표시) / B 경로 숨김 / C 가입 여부도 숨김(이메일 인증 필요). 이유: 가입 경로 노출을 줄이면서 다음 행동은 안내, 로그인 실패 메시지 정책(TC-43)과 일관. 소셜 콜백 ACCOUNT_EXISTS의 provider 전달(명세 135행)도 함께 맞출 것
+관련: #15 (같은 원칙을 로그인 실패 문구에 적용)</t>
         </is>
       </c>
       <c r="N64" s="28" t="inlineStr">
@@ -6764,7 +6765,7 @@
         <is>
           <t>근거: 명세 390행 화면 data-testid signup-password-confirm-error (불일치 시 동작을 적은 문장은 없음)
 QA가 codegen 녹화 후 직접 다듬어 자동화 (tests/ui/my-tests.spec.ts). 기대값을 일부러 틀리게 바꿔 실패하는 것 확인
-Claude 리뷰 반영 (QA 수정): DB에서 계정 0건 확인 추가. 가입 API에는 비밀번호 확인 필드가 없어 요청이 나갔다면 계정이 생겼을 것 → 0건이면 "가입 요청 안 나감"과 "계정 생성 안 됨"을 둘 다 확인하는 셈
+Claude 리뷰 반영 (반영 여부는 QA 판단, 수정 코드는 Claude 작성): DB에서 계정 0건 확인 추가. 가입 API에는 비밀번호 확인 필드가 없어 요청이 나갔다면 계정이 생겼을 것 → 0건이면 "가입 요청 안 나감"과 "계정 생성 안 됨"을 둘 다 확인하는 셈
 고정 이메일(tc71@test.com)은 유지: 테스트 DB가 실행마다 초기화되고, 계정이 잘못 생기면 0건 확인에서 바로 실패로 드러남</t>
         </is>
       </c>
@@ -7262,11 +7263,10 @@
         <is>
           <t>근거: 명세 192행 「소셜 가입 계정은 비밀번호가 없어 항상 401」
 관련: TC-53(이메일 가입 주소로 구글 로그인), TC-63(구글 가입 주소로 이메일 가입)의 반대 방향
-2026-10-13 수동 확인: 기대결과 401은 충족. 일반 실패 문구만 나와 소셜 가입 사용자가 로그인 방법을 알기 어려움 → 개선 제안 #15 (계정별 문구 대신 모든 실패에 같은 소셜 로그인 안내). 실행결과는 자동화 작성 후 기록
+2026-10-13 수동 확인: 기대결과 401은 충족. 일반 실패 문구만 나와 소셜 가입 사용자가 로그인 방법을 알기 어려움 → 개선 제안 #15 (계정별 문구 대신 모든 실패에 같은 소셜 로그인 안내)
 QA가 codegen 녹화 후 직접 다듬어 자동화 (tests/ui/my-tests.spec.ts). 기대값을 일부러 틀리게 바꿔 실패하는 것 확인
 영역은 API이나 UI로 자동화: 화면 로그인도 같은 API를 거치고, login-error의 data-code로 INVALID_CREDENTIALS 확인
-관련 개선 제안 #15 (일반 실패 문구만 나와 로그인 방법을 알기 어려움)
-Claude 리뷰 반영 (QA 수정): 카카오 버튼 href가 채워질 때까지 기다린 뒤 클릭 (처음엔 href="#", TC-53과 같은 문제)</t>
+Claude 리뷰 반영 (반영 여부는 QA 판단, 수정 코드는 Claude 작성): 카카오 버튼 href가 채워질 때까지 기다린 뒤 클릭 (처음엔 href="#", TC-53과 같은 문제)</t>
         </is>
       </c>
       <c r="N78" s="28" t="inlineStr">

</xml_diff>